<commit_message>
Lambda 2023-11-10 TMS 物流产品联调
</commit_message>
<xml_diff>
--- a/erp-server/erp-server-plm/src/main/resources/excel/logisticsProductTemplate.xlsx
+++ b/erp-server/erp-server-plm/src/main/resources/excel/logisticsProductTemplate.xlsx
@@ -11,6 +11,9 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$M$1</definedName>
+  </definedNames>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
@@ -26,10 +29,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>中文英文名</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>报关型号</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -79,6 +78,10 @@
   </si>
   <si>
     <t>税率</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>英文报关名</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -442,50 +445,55 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M1:M1048576">
+      <formula1>"拆分申报,合并申报"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>